<commit_message>
Fixed and distance to and from
</commit_message>
<xml_diff>
--- a/Trip_Data_Store/Jewish_Home_Sample.xlsx
+++ b/Trip_Data_Store/Jewish_Home_Sample.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kshema/python/Four-Line-Travels/Trip_Data_Store/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FCECDBEE-D2BB-ED4F-AB6E-41E0F6FB751C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E237E211-CE42-6B49-B5C3-0BF8305E8F29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6460" yWindow="2520" windowWidth="28040" windowHeight="17440" xr2:uid="{AE5D1BB2-5E34-FD46-9363-BB23602A05C7}"/>
+    <workbookView xWindow="3080" yWindow="2440" windowWidth="28040" windowHeight="17440" xr2:uid="{AE5D1BB2-5E34-FD46-9363-BB23602A05C7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -141,11 +141,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -482,9 +491,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A045AF3-5CFA-1A43-B1C1-FDA570DF2BFF}">
   <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" style="6"/>
+    <col min="5" max="5" width="74.1640625" customWidth="1"/>
+    <col min="6" max="6" width="63.1640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="17" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -504,7 +518,7 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="17" x14ac:dyDescent="0.2">
-      <c r="A2" s="2">
+      <c r="A2" s="5">
         <v>1</v>
       </c>
       <c r="B2" s="3">
@@ -524,7 +538,7 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="17" x14ac:dyDescent="0.2">
-      <c r="A3" s="2">
+      <c r="A3" s="5">
         <v>2</v>
       </c>
       <c r="B3" s="3">
@@ -544,7 +558,7 @@
       </c>
     </row>
     <row r="4" spans="1:6" ht="17" x14ac:dyDescent="0.2">
-      <c r="A4" s="2">
+      <c r="A4" s="5">
         <v>3</v>
       </c>
       <c r="B4" s="3">
@@ -564,7 +578,7 @@
       </c>
     </row>
     <row r="5" spans="1:6" ht="17" x14ac:dyDescent="0.2">
-      <c r="A5" s="2">
+      <c r="A5" s="5">
         <v>4</v>
       </c>
       <c r="B5" s="3">

</xml_diff>